<commit_message>
Nightly job search: 1 fresh match (Accenture Full Stack Engineer - GenAI)
Searched 12+ platforms for jobs posted in the last 24 hours matching
Siva Kumar's profile (Lead Full Stack / AI Infrastructure). Only one
listing cleared both the freshness window and the 60% fitness bar:
Accenture's Full Stack Engineer (Generative AI) role in Hyderabad,
posted 2026-09-01. Generated a tailored resume and cover letter and
appended the tracker entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016zn1dQFBu5yPjhAZso4PjH
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,73 @@
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer (Generative AI)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_558</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (on-site)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaqgzvq6ckzx</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>63% Fit</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>JD asks for min 5 yrs specifically in Generative AI (SME/team-lead scope); Siva has ~14 months hands-on GenAI (TokenSight AI gateway) on top of 9 yrs overall full-stack + cloud experience, which covers the full-stack/cloud/agile requirements well but is short on GenAI-specific tenure.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches (Verisk Lead AI Engineer, Paktolus FDE)
Both posted within the last 24 hours (2026-09-08) and scored >=60% fit.
Excluded Webflow Senior FDE (Austin, TX) - requires US work authorization,
not eligible for India-based remote. Other platforms (Naukri, LinkedIn,
Instahyre, Hirist, Cutshort, Wellfound) returned no listings with a
confirmable posting date inside the 24h window this run - WebFetch is
blocked for those domains in this environment, so their dates couldn't be
verified per the freshness rule.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G1Bzft6FYbyAnP6fkf2EY1
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -769,6 +769,140 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignite Insurance Systems (Verisk)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lead AI Engineer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_1597</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (on-site)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aagqrsk46bkw</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>74% Fit</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Strong match: 9 yrs full-stack/backend incl. Lead title vs 8+ yrs required; TokenSight (LLM gateway, cost/latency optimization, OpenTelemetry observability, Presidio for responsible-AI data handling) maps directly to the JD's core asks. Gaps disclosed honestly: ~14 months hands-on GenAI vs 2-year minimum, and no hands-on multi-agent orchestration / MCP tooling yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paktolus</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_1534</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aav8ckmdsjvx</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>64% Fit</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Moderate fit: 9 yrs vs 7+ yrs required, strong Python/FastAPI/AWS/Docker/K8s and LLM API integration/prompt engineering overlap via TokenSight. Key gap: JD wants 3+ yrs in formal external customer-facing implementation/consulting roles and enterprise CRM/ERP/HRMS integration experience, which Siva does not have (his stakeholder work has been internal); LangChain/LlamaIndex and vector-DB/RAG hands-on also not on his profile. Disclosed honestly in cover letter.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 1 fresh match (NewRocket Senior/Lead FDE - Anthropic, Boston)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DcsQVHLG6zrHs3k2FmG9AJ
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,73 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NewRocket (AI Foundry — Anthropic partner)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Senior/Lead Forward Deployed AI Engineer - Anthropic (US East)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_1804</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Boston, MA (Remote with ~70% travel)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa4zcptwkbtk</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>64% Fit</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>New requisition (distinct Job ID/posting from the Sept 3 NewRocket FDE listing already tracked) for the same AI Foundry/Anthropic program, but this one requires 8+ yrs (Siva has 9, a cleaner match than the prior 5-8 yr req) and lists heavier travel (~70% vs ~25%). Same core gaps as before: customer-facing/consulting delivery is new territory (his background is internal product engineering), no hands-on Anthropic/Claude API experience yet, and eligibility/visa for a US-based, high-travel role from India is unconfirmed in the JD — flagged honestly in the cover letter. Two sibling reqs for the same program also posted Sept 10 (Seattle JOBSEARCH_1802, Atlanta JOBSEARCH_1805) with near-identical JD text — skipped as duplicates of this one rather than generating triplicate materials.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches (KONG Staff FDE, Coalition Staff Security Eng)
Both posted within the last 24 hours per Indeed API, Fitness >= 60%.
Generated tailored resume + cover letter for each; tracker updated.
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -970,6 +970,140 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KONG</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Staff Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_1934</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ (on-site, not marked remote)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aajzl86tvjmc</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>62% Fit</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Strong domain match: Kong is 'the AI Connectivity Company' building an API/AI gateway; Siva owns TokenSight, an enterprise AI gateway (FastAPI/ClickHouse/Redis/OpenTelemetry/Presidio) at CloudAngles -- same connectivity-layer problem. 9 yrs vs 8+ yrs required fits. Gaps disclosed honestly: no formal external customer-facing/consulting delivery experience (internal product engineering background only), and no hands-on Terraform/Ansible/Helm (has Docker/K8s/CI-CD instead). Posting lists Phoenix, AZ without a remote tag -- flagged to candidate as a relocation/remote-arrangement question before applying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Coalition Inc.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer, Security Engineering</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_1941</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa849jnqmmp9</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>64% Fit</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Good skills match: Python/FastAPI, TypeScript/Node.js, React (a plus), API design, and AI-assisted workflows all line up with Siva's TokenSight work. Staff-level IC scope matches his Lead-level ownership. Gap disclosed honestly: no dedicated cybersecurity-domain background -- his security-adjacent experience is Presidio PII redaction and PCI-DSS fintech integrations (Razorpay/Stripe/PayU), not core security engineering. Salary listed in US bands; remote-from-India eligibility is unconfirmed in the JD, flagged to candidate.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 9 fresh matches found (Lenovo, Target, IFS, GeneralMind, Beacon Biosignals, LawPro.ai, Ocean Infinity, Analytica, DEMECAN)
All postings verified within last 24h via Indeed API. No fresh matches found in Hyderabad/Remote India this run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QYK53pF8bYp8deR5aGr5E8
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1104,6 +1104,609 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lenovo</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Frontend Engineer, AI Platform and User Experience (posted as: Web Front-End Developer – Agentic AI Applications)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2476</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Morrisville, NC (hybrid, 3 days on-site/2 remote)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aanfg864t8ht</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>88% Fit</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Excellent match: JD confirms React/TS frontend for Agentic AI applications, prompt-engineering-aware UX, RESTful/FastAPI backend integration, Redux/Zustand-style state management -- near-exact overlap with Siva's TokenSight dashboard work (React/Next.js on an LLM/AI gateway, Redux Toolkit, FastAPI backend). Gaps disclosed honestly: no Storybook/Zustand specifically (has Redux Toolkit/Saga instead); hybrid on-site in Morrisville, NC needs relocation/visa sponsorship from India -- flagged in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lead Engineer – Platform AI – Cloud and Compute (full stack)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2737</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Brooklyn Park, MN (on-site)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aacwthzylmtk</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>85% Fit</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Strong match: Lead Engineer role explicitly covers full-stack + platform AI + cloud/compute (Kubernetes, containers, observability) leadership, matching Siva's Lead title, Docker/K8s, and OpenTelemetry observability work on TokenSight. Gap disclosed: JD lists Java/Go/Kotlin as example stacks; his production languages are Python/Node/TypeScript -- transferable but not an exact stack match. On-site Minnesota relocation/visa unconfirmed in posting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IFS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Senior Lead Agentic AI Engineer – Construction &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2676</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Staines-upon-Thames / London, UK (on-site/hybrid)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa2cpbtdvk2x</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>85% Fit</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Strong match: small-team lead role shipping full-stack features with agentic architectures/RAG on Kubernetes, AI-assisted development (Claude Code/Cursor), forward-deployed customer engagement -- mirrors Siva's TokenSight LLM-gateway ownership and his interest in FDE-track roles. Gaps disclosed honestly: no formal external customer-facing consulting background yet (his stakeholder work has been internal), no formal RAG-pipeline build experience; UK Skilled Worker visa sponsorship unconfirmed in posting -- flagged in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GeneralMind</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lead Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2683</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Berlin, Germany (on-site)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aahb8lhdzc4v</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>75% Fit</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Moderate-strong match: title is an exact match to Siva's target role (Lead Full Stack Engineer); company appears to be a small AI-product company (employs AI Platform Engineers and Staff Frontend Engineers per LinkedIn), aligning with his AI-gateway + React/Next.js background. Caveat: full JD text was not available via search (title/company-only match, disclosed honestly in the cover letter); Berlin on-site would need EU work authorization -- EU Blue Card raised as the open visa question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Beacon Biosignals</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer, Data Platform</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2568</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Boston, MA (fully remote, anywhere in the US)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aad6bwgfxgkb</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>72% Fit</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Good match: Staff-level backend/data-platform role (7+ yrs incl. 3+ yrs on data platforms; Postgres, event-driven pipelines, GraphQL, hand-written SQL) lines up with Siva's ClickHouse/Redis/Postgres backend work on TokenSight and his 9 years experience. Gaps disclosed: no direct Kafka experience (has WebSocket/streaming-adjacent work instead); health-tech/biosignals is a new domain; remote-in-US eligibility from India is unconfirmed -- flagged in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LawPro.ai</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2470</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aakzxbvzt6nn</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>65% Fit</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Moderate match: small legal-AI startup building LLM evaluation frameworks/pipelines for a legal-focused AI analytics platform -- conceptually close to Siva's TokenSight LLM-observability and cost/quality-optimization work. Gaps disclosed: posting states employees work from home from any US state, suggesting US residency/work authorization may be expected (unconfirmed for India-based applicants, flagged in cover letter); no legal-domain background; "AI Engineer" (not Lead) title may be a level below his current scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ocean Infinity</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Engineering Tech Lead (Full Stack)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2747</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>London, UK (on-site)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaf6kdv66v7m</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>64% Fit</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Moderate match: tech-lead-level full-stack ownership matches Siva's Lead scope, and the React/TypeScript frontend portion of their stack lines up directly. Major gap disclosed plainly in materials: their backend in this JD family is built on .NET/Java/microservices, which isn't in Siva's stack (Python/FastAPI/Node.js) -- framed as a real open question, not glossed over; maritime-robotics domain is also new to him. UK visa sponsorship unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Analytica</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Lead Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2738</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Bethesda, MD (on-site)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aay9ftlg244g</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>60% Fit ⚠️ STRETCH</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Stretch match: title matches (Lead Full Stack Engineer) and their full-stack work (secure, scalable enterprise applications) fits his production experience, incl. PCI-DSS regulatory-constraint experience at Altimetrik. Major gap flagged prominently: Analytica is a public-sector consulting firm serving health/civilian/national-security missions -- roles like this commonly require US citizenship or security-clearance eligibility, unconfirmed and likely a hard blocker applying from India. Verify eligibility before investing further time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DEMECAN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lead Engineer Telemedizin-Plattform (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2829</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Berlin, Germany (on-site)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aabggcdnhz7l</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>67% Fit ⚠️ STRETCH</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Stretch match: "Lead Engineer" for a telemedicine platform matches his lead/full-stack/platform scope conceptually. Major gap flagged prominently and honestly in the cover letter: the "(m/w/d)" tag and German-market context strongly suggest German-language fluency is required, which Siva does not have -- he does not claim it, and flags this as the primary open question before proceeding.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 3 fresh matches posted in last 24h (Coalition Frontend Engineer, MongoDB FDE, Teradata Sr Full Stack AI Platform)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145v9P2KZ9ostifDK6chub5
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1707,6 +1707,207 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Coalition Inc.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Frontend Engineer, Underwriting</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_2999</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aanlbgmwzdyv</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>80% Fit</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Strong match: React/TypeScript frontend for a data-heavy application (underwriting workbench) with dedicated interfaces for AI-assisted workflows -- near-exact overlap with Siva's TokenSight dashboard work (React/Next.js on an LLM/AI gateway, Redux Toolkit state management, REST API integration, AI-driven UX surfacing cost/prompt signals). JD asks for 2+ yrs (Siva has 9, comfortably exceeds). Gaps disclosed honestly: no insurtech/cybersecurity domain background, and his observability tooling is OpenTelemetry-based rather than Sentry/Datadog specifically. Different distinct role/Job ID from the Coalition Staff Security Engineer listing already tracked (Sept 12) -- separate application, not a duplicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer, Industry Solutions</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3069</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Toronto, ON (remote-based, regular travel to partner sites)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aactq4qwdpdh</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>68% Fit</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Good match: 5+ yrs backend required (Siva has 9), strong coding ability across Python/FastAPI and Node.js/TypeScript, hands-on MongoDB (listed in his stack alongside ClickHouse/Redis/Postgres on TokenSight), APIs, containers (Docker/K8s), and cloud deployment all line up. Gaps disclosed honestly: no formal embedded/forward-deployed partner-engineering experience (closest analogue is integrating third-party payment gateways into an existing PCI-DSS codebase at Altimetrik), and no hands-on database-migration/CDC experience. Role is remote-based out of Toronto with regular on-site partner travel -- Canada work authorization/visa sponsorship and travel logistics unconfirmed in the JD, flagged to candidate before applying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Teradata</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sr Full Stack Engineer - AI Platform</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3009</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (on-site)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aasf6nc4tjz8</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>62% Fit</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Moderate match: multi-tenant cloud-platform console dashboard for an AI platform (Teradata Autonomous Knowledge Platform) closely mirrors Siva's TokenSight dashboard ownership (usage/cost/monitoring UI on a FastAPI backend, AWS-deployed). 5+ yrs required, Siva has 9. Major gap flagged prominently and honestly: the JD's primary frontend stack is Angular/Angular Material, while Siva's production frontend experience for the last several years has been React/TypeScript (Angular was only his stack at an earlier role, 2018-2019) -- disclosed as a real transition, not a checkbox already met. Same city as candidate (Hyderabad) -- no relocation needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 4 fresh matches posted in last 24h (Ookla, HighLevel, Resourceful Talent Group, Capgemini)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y3UC96AxKriCgsUXXo6Yep
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T21"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,274 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ookla (an Accenture company)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Developer - Downdetector Connect</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3161</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>London, UK (on-site/hybrid, comp listed in GBP)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aar2tbb64l8q</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>78% Fit</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Strong match: full-stack role building React/Redux interfaces over a Python/FastAPI backend handling high-volume time-series telemetry, with AI-driven 'Observe-Think-Act' automation -- closely mirrors Siva's TokenSight ownership (FastAPI/ClickHouse/Redis backend + React/Next.js frontend + AI-driven cost-signal UX). 9 yrs vs 5-8 yrs required fits well. Gaps disclosed honestly: no explicit Terraform (has Docker/K8s instead), and telecom/network-monitoring is a new domain. London on-site listing with GBP comp -- relocation/visa sponsorship from India unconfirmed, flagged in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HighLevel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Senior Software Development Engineer (Agency Success)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3184</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Remote (remote-first, 10+ countries)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aajysylpppwj</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>82% Fit</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Excellent match: JD explicitly lists ClickHouse alongside MongoDB and Redis -- exactly Siva's TokenSight data stack -- plus Node.js/TypeScript backend (his MERN-era stack at Altimetrik/Pegasystems) and LLM/AI-assisted workflow exposure (TokenSight's AI-driven cost signals). React accepted (Vue preferred, not required). 9 yrs comfortably clears the 4+ yr bar. Gaps disclosed honestly: no hands-on Elasticsearch or Kafka/Pub-Sub (WebSocket/Redis-based patterns instead), and observability tooling is OpenTelemetry-based rather than Grafana/Prometheus/Sentry specifically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Resourceful Talent Group (fintech client, via agency)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Senior Full-Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3169</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Berlin / Fully Remote (EST hours)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aadj6gn4cdj9</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>68% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Good technical match: React/TypeScript + Node.js/TypeScript full stack, hands-on PostgreSQL (via TokenSight), and direct fintech/payments domain experience (PCI-DSS, Razorpay/Stripe/PayU at Altimetrik) map closely to this role's ACH/reconciliation/compliance asks; comfortable using Claude/AI coding tools as required. MAJOR GAP flagged prominently and honestly: posting requires 'Strong English and Russian communication skills' -- Siva does not speak Russian, disclosed plainly in the cover letter as a likely hard blocker to verify with the recruiter before investing further time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Agentic GEN AI Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3222</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka (on-site)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa9k8dbwvfhr</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>61% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Moderate/borderline match: Python + React experience comfortably exceeds the 3+ yr requirement, and AWS/Docker transfer directly. MAJOR GAP disclosed honestly: JD specifically wants 2+ yrs building RAG-based chatbots/Agentic AI systems -- Siva's LLM work is AI-gateway observability/cost optimization (TokenSight), not RAG-pipeline or chat-agent building, a real skills gap not a checkbox already met. Also no Terraform or DynamoDB (has Docker/K8s and Postgres/Mongo/ClickHouse/Redis instead). Additionally this is a 3+ yr IC req vs Siva's Lead-level/9-yr profile -- worth clarifying actual seniority/scope before applying. Same city as candidate (Hyderabad-&gt;Bangalore) -- no cross-country relocation needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 3 fresh India matches posted in last 24h (JPMorganChase, UST, Technical Lead contract)
Abroad Indeed search hit API rate limiting; India web boards (Naukri, LinkedIn,
Instahyre, etc.) and remote/startup boards (Wellfound, career pages) blocked by
this session's egress policy. Continuing to work through the rate limit for
abroad results before finalizing the run's report.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019g43HagC5RxMHkKNDTrADj
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2176,6 +2176,207 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>JPMorganChase</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Lead Software Engineer- Python Full Stack Development (Python, Django &amp; React)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3866</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka (on-site)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aamjjn9m2f72</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>84% Fit</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Strong match: 9 yrs vs 5+ required, Python + React full-stack lead role at a large enterprise with explicit financial-services domain (Altimetrik fintech/PCI-DSS experience maps directly). JD's ask to drive team adoption of AI-assisted engineering practices lines up with Siva's TokenSight work setting internal standards for validating LLM-generated output. Gap disclosed honestly: production Python framework has been FastAPI, not Django -- patterns transfer but no direct Django experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>UST</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lead I - Software Engineering (Senior Front-End &amp; API Developer)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3937</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aakp7dsrmxsx</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>81% Fit</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Strong match: React/TypeScript dashboard and workflow-UI work over a Python API layer, with monitoring/incident-response built in -- near-exact overlap with Siva's TokenSight frontend (React/Next.js/Redux Toolkit over FastAPI, OpenTelemetry-driven monitoring). 9 yrs comfortably clears the 5+ yr bar. Gaps disclosed honestly: no specific GitHub Copilot usage and no hands-on MCP protocol experience, though LLM API integration/prompt engineering is part of his daily TokenSight work. Duplicate listing also seen as JOBSEARCH_4000 (same posting) -- tracked once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Technical Lead - Full Stack Development (company undisclosed, via hiring/consulting account)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Technical Lead - Full Stack Development</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_3917</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gopanpalli, Telangana / Hyderabad hub (Hybrid, Contract up to Rs24L/yr)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaxv8xfpyjs9</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>62% Fit</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Moderate match: excellent alignment on the AI/LLM-infrastructure and responsible-AI side (LLM API integration, Presidio for PII/data-privacy, OpenTelemetry observability -- directly parallels TokenSight) and on distributed-systems/technical leadership (9 yrs vs 8-12 required). MAJOR GAP disclosed plainly and prominently: JD requires Expert Go and Red Hat OpenShift + Terraform/Ansible, none of which are in Siva's stack (Docker/Kubernetes instead) -- flagged honestly in the cover letter rather than fabricated. Contract role, not full-time.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tidy company/role field split for undisclosed Technical Lead contract listing
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019g43HagC5RxMHkKNDTrADj
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -2318,12 +2318,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Technical Lead - Full Stack Development (company undisclosed, via hiring/consulting account)</t>
+          <t>Undisclosed Client (via hiring/consulting account)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Technical Lead - Full Stack Development</t>
+          <t>Technical Lead – Full Stack Development</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">

</xml_diff>

<commit_message>
Nightly job search: 3 fresh matches posted in last 24h (GE Aerospace, Rebud Cyber, IFS FDE)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DmoYQQ8YXv6FAm9nrVsxUE
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T28"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2377,6 +2377,207 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GE Aerospace</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Principal Software Engineer (AI-Powered Full Stack, CES Business Intelligence)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_4391</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Remote (US) — legally-authorized-to-work-in-US required per posting</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aadzkdpb9tjb</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>75% Fit</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Strong match: Principal/senior-IC full-stack role explicitly built around embedding AI/LLM APIs and agentic workflows into production apps -- directly mirrors Siva's TokenSight ownership (FastAPI/React AI gateway, LLM integration, cost optimization, mentoring). 9 yrs vs 8+ required fits. Gaps disclosed honestly: no MCP-server building or knowledge-graph/ontology modeling specifically, data platform is ClickHouse/Postgres rather than Databricks/Snowflake, and no supply-chain/manufacturing domain. MAJOR FLAG: posting states GE Aerospace will only employ candidates already legally authorized to work in the US -- Siva does not hold this and it's disclosed upfront in the cover letter rather than glossed over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Rebud Cyber</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_4395</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Remote — posting requires US-based with Eastern time overlap</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aazt2qt8tvbq</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>82% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Excellent technical match: expert React/Next.js (App Router)/TypeScript, deep Postgres, real-time WebSocket features, and third-party API integration (OAuth/rate-limits/retries) all map directly to Siva's TokenSight dashboard work and Altimetrik payment-gateway integrations (Razorpay/Stripe/PayU under PCI-DSS). 9 yrs vs 5+ required comfortably clears the bar. MAJOR GAP flagged prominently and honestly: posting explicitly requires the candidate be US-based with substantial Eastern time overlap -- Siva is Hyderabad-based, a real mismatch against the posting as written, disclosed directly in the cover letter rather than talked around.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IFS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer – Aerospace and Defense</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_4486</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Ottawa, ON, Canada (on-site/embedded with customers)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaxvnn7m7mcp</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>68% Fit ⚠️ STRETCH</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Moderate match: full-stack breadth (backend/APIs/web front ends) and AI-in-production experience (LLM API integration, prompt engineering) line up with the JD's 'strong plus' AI criteria and Siva's TokenSight ownership; senior-level autonomy matches his Lead scope. MAJOR GAPS flagged prominently and honestly: no forward-deployed/customer-embedded delivery experience (his stakeholder work has been internal, not on customer sites), no aerospace/defense/MRO domain background, and Canadian work authorization plus likely citizenship/security-clearance expectations for defense-sector client work are unconfirmed -- flagged as open questions to verify before investing further time, not glossed over.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (Luxoft, Nexus One)
Luxoft Front-End Developer (Hyderabad, 88% Fit) and Nexus One Forward
Deployed Engineer (Atlanta, 63% Fit, visa/location gap flagged) both
posted 2026-09-22/23. Tailored resume + cover letter generated for
each, tracker updated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185icntVToBp4giz93SiJAv
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:T33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2578,6 +2578,140 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Luxoft</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Front-End Developer (React, Micro Frontends)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_4546</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aatnz4xpc9qd</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>88% Fit</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Excellent match: direct React/TypeScript + Micro Frontend (Webpack Module Federation) experience from GlobalLogic maps 1:1 onto the JD's core requirement. 9 yrs vs 6-9 yr band is a slight overshoot at the top end, which helps against the JD's explicit ask for mentoring and leading technical initiatives. Banking/financial-services domain exposure (Altimetrik, PCI-DSS payment gateway integrations) directly covers the JD's 'nice to have' enterprise/regulated domain line. Hyderabad-based, no relocation needed. Only soft gap: last two years have been Lead-level full stack rather than pure front-end IC work, disclosed in the cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nexus One</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_4540</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (customer-site travel expected)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aayzsnmhxrvc</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>63% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Moderate match: strong production ownership of an AI/data platform (TokenSight -- FastAPI, ClickHouse, Redis, OpenTelemetry) and Kubernetes/Python fundamentals line up with the JD's engineering bar, and PCI-DSS payment-gateway integration work at Altimetrik is a real analogue for integrating with a regulated customer's existing stack. 9 yrs comfortably clears the 6+ yr requirement. MAJOR GAPS disclosed plainly: no post-sales/customer-embedded FDE experience (internal product engineering only), no hands-on Spark/Trino/Iceberg/Kafka/Airflow/Terraform, and the posting is based in Atlanta with customer-site travel and no stated visa sponsorship or remote-from-India path -- work authorization is a real open question, flagged upfront in the cover letter rather than glossed over.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 3 fresh matches posted in last 24h (ThinkDigits, HighLevel, Ameriprise)
ThinkDigits Senior Full Stack Developer (Hyderabad, 80% Fit), HighLevel
Staff Engineer - Platform Frontend (Remote, 74% Fit), and Ameriprise
Financial Lead Full Stack Developer (Noida, 68% Fit) all posted
2026-09-24. Tailored resume + cover letter generated for each, tracker
updated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ihPnEcEyeZdnReYtYamNa
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2712,6 +2712,207 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ThinkDigits</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Developer (In-House Product)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100060</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Madhapur, Hyderabad, Telangana (on-site, 5 days/week)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa4kywxbmxl6</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>80% Fit</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Very strong stack match: React/TS + Python/FastAPI + Postgres + AWS/Azure mirrors TokenSight exactly; 6+ yrs required vs Siva's 9. In-office in Madhapur, Hyderabad — no relocation needed. Gap: no Azure experience (AWS only); company name not disclosed in listing (early-stage/in-house product team).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HighLevel</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Staff Engineer - Platform Frontend</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100084</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Remote (remote-first, global)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aacrv89dq4lm</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>74% Fit</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Strong architecture match: 9+ yrs frontend required = exact fit; micro-frontend/module federation ownership from GlobalLogic directly matches the core ask. Gap: stack is primarily Vue 3, Siva's production depth is React (JD explicitly welcomes React/Angular/Svelte backgrounds willing to go deep on Vue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ameriprise Financial</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Lead Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100129</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh (hybrid, 3 days/week office)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aatjymb8r6yb</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>68% Fit</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Strong skills + domain match: Python/FastAPI, React, AWS mirrors current stack; fintech/PCI-DSS background from Altimetrik maps to Asset Management domain; 7+ yrs required vs 9, Lead title matches. Gaps: Noida location requires relocation (Siva is Hyderabad-based), no AWS certification, no Terraform.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (Cribl, OpenLoop Health)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MYCtXACg4tf71LajevEJAH
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2913,6 +2913,140 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cribl</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer, Agentic Tools</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100757</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>San Francisco, CA (remote-first, #LI-Remote)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aakl6nj9vdxs</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>72% Fit</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Strong platform match: role is building shared agent runtime, observability, and guardrails for agentic systems other teams depend on -- directly analogous to Siva's TokenSight ownership (FastAPI/ClickHouse/Redis AI gateway, OpenTelemetry tracing, Presidio PII redaction, 60-70% cost cut, React/Next.js dashboards on top). Strong Node.js/TypeScript + React background (9 yrs) lines up with the team's primary stack. Gaps disclosed honestly: no hands-on job-orchestration (Temporal) or developer-facing coding-agent harness building specifically, and the posting lists San Francisco with a remote-first note -- India-remote eligibility is unconfirmed and flagged as an open question rather than assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>OpenLoop Health</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100641</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Des Moines, IA (Remote within the United States)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aawtv6ff6frf</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>66% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Moderate-strong technical match: integration-engineering core (API design, webhooks, idempotency, rate limits) maps well onto Siva's PCI-DSS payment-gateway integrations at Altimetrik (Razorpay/Stripe/PayU), and TokenSight's production LLM-in-the-loop observability/evaluation work covers the 'build with AI agents, verify what they produce' ask. 9 yrs comfortably clears the 5-15+ yr band (role is leveled Senior/Staff/Sr-Staff during process). MAJOR GAP flagged prominently and honestly: no customer-embedded/client-facing FDE delivery experience (internal product work only), no healthcare/EHR domain, and the posting is explicitly remote-within-the-United-States with no stated sponsorship -- Siva is Hyderabad-based without current US work authorization, disclosed directly in the cover letter rather than glossed over.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 4 fresh matches posted in last 24h (Qualminds, Neuehealth, Commonwealth Bank, Okta)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NbR5jwovkHKRgqkFaMBRTT
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T38"/>
+  <dimension ref="A1:T42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3047,6 +3047,274 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Qualminds Technologies</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Lead Engineer – Agentic AI</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100914</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aarfvgjwghbs</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>70% Fit</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Strong infra/guardrails match: TokenSight's AI gateway (FastAPI/ClickHouse/Redis, OpenTelemetry tracing, Presidio PII redaction, LLM cost optimization) covers the observability/guardrails backbone this role needs, and 9 yrs clears the 8+ yr bar. Python/TypeScript, FastAPI, and React/Next.js line up directly with the stated stack. GAP disclosed honestly: no hands-on multi-agent orchestration (LangGraph, OpenAI/Claude Agents SDK) or realtime voice AI pipelines specifically -- the role's core ask is architecting multi-agent systems, which is a step beyond gateway/observability work. Hyderabad-based, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Neuehealth</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100846</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Minneapolis, MN (Work-from-home; TX/MN/FL preferred)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa279lprbl2q</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>65% Fit</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Moderate-strong technical match: production LLM/AI engineering (TokenSight's observability, PII redaction via Presidio, cost/usage monitoring) maps onto the JD's RAG/evaluation/guardrails/human-in-the-loop asks, and regulated-environment delivery (PCI-DSS at Altimetrik) is a real analogue for HITRUST-aligned healthcare AI, even without healthcare domain itself. 9 yrs clears the 5+ yr requirement. GAP flagged prominently: no healthcare/PHI domain experience, and the posting is a US work-from-home role with TX/MN/FL preferred and no stated sponsorship -- Siva is Hyderabad-based without confirmed US work authorization or remote-from-India eligibility, flagged as an open question rather than glossed over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Commonwealth Bank of Australia</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100927</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka (Manyata Tech Park)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aanmrxwcn6j8</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>73% Fit</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Strong stack match: Python and React.js are both mandatory and are Siva's core TokenSight stack, with AWS and AI/agent-workflow experience (LLM gateway, OpenTelemetry, Presidio) directly relevant to the JD's 'AI-powered, agent-driven systems' ask. PCI-DSS payment-gateway work at Altimetrik is a reasonable secure-coding analogue for a data-security team, though not a direct cybersecurity domain background. Gap: 9 yrs vs. 10-14 yrs required (slightly under), and no dedicated cybersecurity/data-security team experience. Requires relocation from Hyderabad to Bangalore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Okta</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer - Full Stack</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_100928</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka (#LI-Hybrid)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aar2dc68whsq</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>72% Fit</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Strong match on experience band (8+ yrs required, 9 yrs held) and stack: hands-on Node.js/TypeScript backend from Altimetrik and Pegasystems MERN work, plus React frontend leadership from GlobalLogic and the TokenSight dashboards -- covers the JD's backend-expertise-plus-frontend-familiarity ask well. Recent AI-gateway/OpenTelemetry work loosely aligns with Okta's stated 'secure AI as well as human identity' direction. Gap: no IAM/identity protocol experience (OAuth, OIDC, SAML) -- the role's core domain. Requires relocation from Hyderabad to Bangalore.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 3 fresh matches posted in last 24h (Diebold Nixdorf, Mastercard FDE, Google AI Platform)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A3B5K33hJcjvFeD7QPKfeS
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T42"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3315,6 +3315,207 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Diebold Nixdorf</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Lead Fullstack AI Development Engineer</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101299</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aav9zlvd2m87</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>80% Fit</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Strong full-stack-AI match: role is architecting AI product suites end-to-end (front end, orchestration APIs, DevOps) -- directly mirrors Siva's TokenSight ownership (FastAPI/ClickHouse/Redis gateway, React/Next.js dashboard streaming live LLM token responses over WebSockets, OpenTelemetry tracing, Presidio PII redaction). 9 yrs lands inside the 8-12 yr band with 3+ yrs leadership required. React/Next.js/TypeScript and Python backend line up directly. Gap disclosed honestly: no hands-on LangChain/LlamaIndex/PyTorch/TensorFlow or agentic frameworks (AutoGen/CrewAI), and no dedicated vector-database/semantic-search work -- his LLM depth is gateway/observability, not model-orchestration. Hyderabad-based, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lead Forward Deployed Engineer (AI)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101311</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra (relocation from Hyderabad required)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aag4zssngjsz</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>63% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Moderate match on Siva's actual target-role category (Forward Deployed Engineer): Python/SQL fluency, hands-on LLM API integration/prompt engineering, and three years of PCI-DSS-constrained payment-gateway delivery at Altimetrik (Razorpay/Stripe/PayU) map onto Mastercard's regulated, data-sensitive client environment. TokenSight's origin story (scope an ambiguous internal ask into a working prototype, then production system) echoes the role's core PoC-scoping motion. MAJOR GAP disclosed plainly: no formal external client-embedded discovery or pre-sales PoC work -- his scoping experience has been with internal engineering stakeholders only, and the role's defining customer-facing, pre-code discovery motion would be new ground. Requires relocation Hyderabad to Pune.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer, AI Platform</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101320</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa9qb9kqcqb7</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>62% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Moderate match: role's explicit requirement to adopt tracing, logging, and monitoring for agentic workflows is a direct hit against Siva's OpenTelemetry instrumentation of every LLM/agent call in TokenSight, and the 'build AI platform tooling other teams depend on' mandate mirrors his gateway ownership. 9 yrs clears the 5-yr bar comfortably. MAJOR GAP disclosed honestly: the role's core ask is 3 years of hands-on end-to-end ML (model deployment, evaluation, optimization, data processing, debugging) plus simulation-orchestration/multi-agent framework experience -- Siva's production depth is at the LLM-gateway/cost-optimization/observability layer, not the classical ML model lifecycle, which is a real stretch against this specific requirement. Hyderabad-based, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (Cornerstone OnDemand, Optum)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XE3dB5iGghPozAxVgVWNm2
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3516,6 +3516,140 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Principal Forward Deployment Engineer</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101457</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (Office/Field Based)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aazzxtzfp9lc</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>67% Fit</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Strong match on the Forward-Deployed-Engineer target category and AI depth: 6+ yr enterprise deployment bar cleared with 9 yrs, and TokenSight (production LLM/agentic gateway, OpenTelemetry tracing, Presidio guardrails) covers the '1-2 yrs deploying GenAI/Agentic Frameworks in production' ask directly. Three years of PCI-DSS payment-gateway integration work at Altimetrik (Razorpay/Stripe/PayU) is a reasonable analogue for the enterprise-integration/REST-API pattern this role needs. MAJOR GAP disclosed honestly: no formal external enterprise-customer-facing solutions engineering or pre-sales discovery experience (his deployment work has been for internal engineering stakeholders), and no HRIS/HCM (Workday, SAP SuccessFactors) exposure. Hyderabad office-based role, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Senior Manager, Agentic AI Engineering</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101458</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aatjy4yvmfcz</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>61% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Moderate match, stretch on seniority shape: TokenSight's production agentic/LLM gateway work (OpenTelemetry tracing, cost/usage analytics, Presidio guardrails) maps well onto the role's AI evaluation/scoring/failure-mode-analysis engineering practice, and React/Next.js experience is a direct hit on the preferred full-stack skill. 9 yrs clears the 7+ yr bar. MAJOR GAP disclosed plainly: this is a people-management title requiring 3+ yrs formal engineering management with direct reports -- Siva has led technically as an IC (architecture, delivery ownership, informal mentoring) but has not managed a team, so that would be new ground, not something to oversell. Also no healthcare domain experience and AWS rather than Azure cloud depth. Hyderabad-based, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 1 fresh match posted in last 24h (Avalon Healthcare Solutions AI Engineer)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9WkowWxHtFp9d1ABX7ydS
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3650,6 +3650,73 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Avalon Healthcare Solutions</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101790</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Tampa, FL (Remote-eligible; quarterly travel to Tampa)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aacgj496brdf</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>66% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Moderate match: 8-10 yrs required vs 9 held, senior IC/informal-leadership scope matches Siva's Lead-level profile well, and TokenSight's production LLM-gateway work (OpenTelemetry tracing, Presidio PII redaction, prompt engineering, LLM API integration, per-model cost analytics) maps directly onto the role's evaluation/guardrails/observability practice. Python and Node.js/TypeScript line up with the JD's polyglot backend ask. MAJOR GAPS disclosed honestly: no Rust/GoLang (JD wants both), no hands-on n8n or comparable workflow-orchestration platform, no vector-database/RAG-pipeline build experience specifically, and no healthcare/HIPAA domain background -- PCI-DSS fintech work at Altimetrik is the closest regulated-data analogue. Role is listed remote-eligible with quarterly travel to Tampa, FL -- India-based work authorization/eligibility is unconfirmed in the posting and flagged as an open question before applying, not assumed either way.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: add 2 fresh matches (ServiceNow, Mastercard)
Searched for roles posted within the last 24 hours only, per the
nightly pipeline's strict freshness rule. Added tailored resume +
cover letter for each match scoring >=60% fitness, updated the tracker.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EEY5M9UxJV3CmQtvoYFVik
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3717,6 +3717,140 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer (AI-Native Platform)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_101938</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (on-site)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aajtbfd8yjlq</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>73% Fit</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>8+ yrs required, Siva has 9; strong overlap on LLM API integration, OpenTelemetry observability/tracing, Presidio-style guardrails, Python/Node backend, React frontend, Docker/K8s/CI-CD. Gap disclosed honestly: role wants hands-on RAG/retrieval, embeddings/vector-store debugging, and formal eval-harness/golden-dataset building (LangChain/LlamaIndex) -- Siva's depth is at the LLM-gateway/cost/tracing layer, not that eval-infrastructure layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Senior Full-Stack Engineer - Open Finance (React, TypeScript, Node &amp; Java)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_102141</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, Maharashtra (on-site)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaxqqxqdts88</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>71% Fit</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>5+ yrs required, Siva has 9; React/TypeScript/Node is an exact match, PCI-DSS fintech/payment-gateway background (Razorpay, Stripe, PayU) at Altimetrik maps directly to the Open Finance domain, and daily Claude/Copilot usage matches the JD's explicit AI-fluency ask. Gap disclosed honestly: Java is a required backend language and Siva's production backend work has been Node.js/Python, not Java. Location is Navi Mumbai (on-site) -- relocation from Hyderabad needed, flagged to candidate.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nightly job search: 1 fresh match posted in last 24h (Optum Senior SWE Lead - React/Python/Cloud/GenAI)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbYKCZJgBZKtDwbqyCzjLn
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:T54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -3845,136 +3845,203 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>BIPB (Keyrus)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_102426</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>Canary Wharf, London, UK (Hybrid 3 days/week)</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aaqthdhycz26</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>68% Fit ⚠️</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
         <is>
           <t>Strong skills/role-category match: production LLM/agentic gateway work on TokenSight (Python, TypeScript, evaluation, Presidio guardrails, OpenTelemetry tracing) maps directly onto the role's 'deliver production-ready AI with guardrails and reliability' ask, and 9 yrs clears the senior/principal band (£72K-£122K). PCI-DSS payment-gateway integration at Altimetrik (Razorpay/Stripe/PayU) is a reasonable analogue for enterprise-integration/security-review work. MAJOR GAP disclosed honestly: no formal external client-facing discovery or consulting history -- his scoping experience has been with internal engineering stakeholders only. Role is hybrid 3 days/week onsite in Canary Wharf, London; relocation/visa sponsorship is NOT addressed in the posting -- flagged as a real open question before applying, not assumed either way.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Prudentia Sciences</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_102429</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>London (UK) / Dublin (Ireland) / Basel (Switzerland) strongly preferred; exceptional US-ET remote considered</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aatvtpm6lnj7</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="3" t="inlineStr">
         <is>
           <t>64% Fit ⚠️</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr">
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R53" s="3" t="inlineStr">
         <is>
           <t>Strong skills overlap: TokenSight's evaluation/guardrails work (Presidio PII redaction, OpenTelemetry tracing, LLM API integration on Python/FastAPI/AWS) directly mirrors the role's 'build evaluations and guardrails so quality is measured, not assumed' mandate; 5+ yr bar cleared comfortably with 9. PCI-DSS fintech integration at Altimetrik is the closest regulated-data analogue. MAJOR GAPS disclosed honestly: (1) no life-sciences/biopharma/clinical-trial/deal-data domain experience at all; (2) the posting explicitly prioritizes London/Dublin/Basel-based candidates, with only an 'exceptional' US-Eastern-Time remote exception -- it does not list an India-based remote path, which is a real eligibility constraint, not just an unconfirmed detail. Flagged plainly so Siva can decide whether it's worth pursuing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer Lead - React, Python, Cloud, Gen AI</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_103026</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa999pnfctr6</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>68% Fit</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Strong stack match: JavaScript/TypeScript/React and Python/API development are both required and are Siva's core TokenSight stack, and hands-on production LLM/GenAI integration (prompt engineering, LLM API integration via TokenSight) directly covers the role's 'integrate LLMs, GenAI services, and intelligent automation' requirement. 9 yrs clears the 7+ yr Agile and 4+ yr cloud bars. MAJOR GAP disclosed honestly: the role's cloud stack is specifically Azure (Azure OpenAI, Azure AI Search, Azure Functions, Terraform) and Siva's cloud depth is AWS, not Azure, with no hands-on Terraform or agent-orchestration frameworks (Semantic Kernel/LangChain/AutoGen) -- those are explicitly required, not just preferred, so this is a real stretch on the cloud-vendor and orchestration-framework specifics even though the underlying GenAI-integration skillset transfers. Hyderabad-based, no relocation needed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (Builders FirstSource Lead Developer AI, Linux Recruit Founding FDE)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G9LtYDkkDj8xRt2trmromL
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T54"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -3979,69 +3979,203 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Optum</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>Senior Software Engineer Lead - React, Python, Cloud, Gen AI</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_103026</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>Hyderabad, Telangana</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aa999pnfctr6</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>68% Fit</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr">
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="inlineStr">
         <is>
           <t>Strong stack match: JavaScript/TypeScript/React and Python/API development are both required and are Siva's core TokenSight stack, and hands-on production LLM/GenAI integration (prompt engineering, LLM API integration via TokenSight) directly covers the role's 'integrate LLMs, GenAI services, and intelligent automation' requirement. 9 yrs clears the 7+ yr Agile and 4+ yr cloud bars. MAJOR GAP disclosed honestly: the role's cloud stack is specifically Azure (Azure OpenAI, Azure AI Search, Azure Functions, Terraform) and Siva's cloud depth is AWS, not Azure, with no hands-on Terraform or agent-orchestration frameworks (Semantic Kernel/LangChain/AutoGen) -- those are explicitly required, not just preferred, so this is a real stretch on the cloud-vendor and orchestration-framework specifics even though the underlying GenAI-integration skillset transfers. Hyderabad-based, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Builders FirstSource</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Lead Developer - AI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_103334</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aayhnzt2jjzf</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>68% Fit</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Strong production-AI match: Python + React/Next.js/TypeScript is an exact stack fit, and 3+ yrs of hands-on Agentic/GenAI production work required is directly covered by TokenSight (LLM gateway, prompt engineering, cost optimization, Presidio guardrails) at CloudAngles. 8-10 yrs required, Siva has 9. MAJOR GAPS disclosed honestly: role's cloud stack is specifically Azure (Azure AI Foundry, Azure OpenAI, AKS) and Siva's depth is AWS; no hands-on LangGraph/LangChain/Semantic Kernel or SAP S/4HANA/ERP-integration background. Posting is USD-salaried US remote with US-specific benefits (401k, ADA) and does not confirm eligibility for India-based remote -- flagged as an open question, not assumed either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Linux Recruit (client undisclosed)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer (Founding)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_103306</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aah8xdmy79pf</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>60% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Strong qualitative fit: role explicitly wants a full-stack engineer who has already shipped AI applications into production and can own ambiguous problems end to end on a small team -- exactly TokenSight's build-and-own profile at CloudAngles. 9 yrs comfortably clears a founding-engineer bar. MAJOR GAP disclosed honestly: posting is London-based (GBP 100k-140k) via a recruiter, with no remote option or visa sponsorship mentioned anywhere -- a real, unaddressed relocation/eligibility question for a Hyderabad-based candidate, flagged plainly rather than assumed either way. Treat as a real stretch worth a quick eligibility check before investing more time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nightly job search: add Talkdesk FDE AI Engineer match (2026-10-23)
Only Indeed-sourced listing confirmed posted within the last 24 hours
this run; WebFetch was unreachable for all other job-board/ATS domains
in this session, so Naukri/LinkedIn/Instahyre/Cutshort/Hirist/Foundit/
Shine/TimesJobs/Glassdoor/Wellfound/WeWorkRemotely/direct-company and
abroad boards could not be freshness-verified and were dropped per the
run's strict 24h rule rather than reported unverified.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bk3V4nQgCg55Vo1PLhyWnX
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T56"/>
+  <dimension ref="A1:T57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -4046,136 +4046,203 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Builders FirstSource</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>Lead Developer - AI</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_103334</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aayhnzt2jjzf</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>68% Fit</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr">
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R55" s="3" t="inlineStr">
         <is>
           <t>Strong production-AI match: Python + React/Next.js/TypeScript is an exact stack fit, and 3+ yrs of hands-on Agentic/GenAI production work required is directly covered by TokenSight (LLM gateway, prompt engineering, cost optimization, Presidio guardrails) at CloudAngles. 8-10 yrs required, Siva has 9. MAJOR GAPS disclosed honestly: role's cloud stack is specifically Azure (Azure AI Foundry, Azure OpenAI, AKS) and Siva's depth is AWS; no hands-on LangGraph/LangChain/Semantic Kernel or SAP S/4HANA/ERP-integration background. Posting is USD-salaried US remote with US-specific benefits (401k, ADA) and does not confirm eligibility for India-based remote -- flagged as an open question, not assumed either way.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Linux Recruit (client undisclosed)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer (Founding)</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_103306</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>London, UK</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aah8xdmy79pf</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I56" s="3" t="inlineStr">
         <is>
           <t>60% Fit ⚠️</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr">
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R56" s="3" t="inlineStr">
         <is>
           <t>Strong qualitative fit: role explicitly wants a full-stack engineer who has already shipped AI applications into production and can own ambiguous problems end to end on a small team -- exactly TokenSight's build-and-own profile at CloudAngles. 9 yrs comfortably clears a founding-engineer bar. MAJOR GAP disclosed honestly: posting is London-based (GBP 100k-140k) via a recruiter, with no remote option or visa sponsorship mentioned anywhere -- a real, unaddressed relocation/eligibility question for a Hyderabad-based candidate, flagged plainly rather than assumed either way. Treat as a real stretch worth a quick eligibility check before investing more time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Talkdesk</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Forward Deployed AI Engineer</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_103568</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aav6x7mzp8g6</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>65% Fit</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Strong skills overlap on Python/TS/JS, prompt engineering, and LLM API integration via TokenSight (AI gateway, cost optimization, OpenTelemetry, Presidio). JD wants 5-7 yrs + 1+ yr Agentic AI (Siva has 9 yrs, ~14-16 months hands-on GenAI) and deep multi-agent system architecture experience, which Siva doesn't have yet (TokenSight is observability/cost-gateway work, not agent orchestration). Main gap: role requires formal external customer-facing consulting/implementation experience; Siva's stakeholder work has been internal only. Comp in USD and remote with no explicit India-remote language -- eligibility flagged to candidate before applying. Disclosed honestly in cover letter.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (SingleStore FDE, Revin Senior/Staff Product Engineer)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175HNdBUBeDWL1yrt9zo1U8
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T57"/>
+  <dimension ref="A1:T59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -4180,69 +4180,203 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Talkdesk</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Forward Deployed AI Engineer</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_103568</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aav6x7mzp8g6</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" s="3" t="inlineStr">
         <is>
           <t>65% Fit</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
         <is>
           <t>Strong skills overlap on Python/TS/JS, prompt engineering, and LLM API integration via TokenSight (AI gateway, cost optimization, OpenTelemetry, Presidio). JD wants 5-7 yrs + 1+ yr Agentic AI (Siva has 9 yrs, ~14-16 months hands-on GenAI) and deep multi-agent system architecture experience, which Siva doesn't have yet (TokenSight is observability/cost-gateway work, not agent orchestration). Main gap: role requires formal external customer-facing consulting/implementation experience; Siva's stakeholder work has been internal only. Comp in USD and remote with no explicit India-remote language -- eligibility flagged to candidate before applying. Disclosed honestly in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SingleStore</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Forward Deployment Engineer</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_104906</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aavnwz6tdq2f</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>63% Fit</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Moderate fit: strong overlap on real-time/distributed data systems (ClickHouse/Redis/Postgres via TokenSight) and production troubleshooting, and 9 yrs is close to the 10+ yrs asked for. Main gap disclosed honestly: role is a formal pre-sales/post-sales solutions-consulting seat with external enterprise customers -- Siva's stakeholder work has been internal only, even though he owns TokenSight end to end. Listing does not confirm remote-from-India eligibility or visa sponsorship (SingleStore has a Bangalore office but this req is listed under US salary bands) -- flagged in cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Revin</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Senior/ Staff Product Engineer (Full Stack)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_105065</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>New York, NY (on-site, 4 days/week)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaxfbtbmpdd6</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>78% Fit</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Strong match: TypeScript/React fluency and end-to-end AI-powered product ownership (TokenSight: backend + FastAPI/ClickHouse + React/Next.js dashboards, measured via usage/cost metrics) map directly onto this product-engineer role's core ask. 9 yrs fits their Senior/Staff band. Gaps disclosed honestly: TokenSight's users are internal stakeholders, not external paying customers, and the home-services/vertical-SaaS domain is new. Role is on-site in NYC 4 days/week -- relocation and work-authorization/visa sponsorship from India is unconfirmed in the posting, flagged clearly in the cover letter.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nightly job search: 2 fresh matches posted in last 24h (Keeper Security Sr. Software Architect, G-P Principal SWE Agentic AI)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175HNd91i8FgwEfcP4uqN9e
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:T61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -4247,136 +4247,270 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>SingleStore</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Forward Deployment Engineer</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_104906</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aavnwz6tdq2f</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>63% Fit</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr">
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
         <is>
           <t>Moderate fit: strong overlap on real-time/distributed data systems (ClickHouse/Redis/Postgres via TokenSight) and production troubleshooting, and 9 yrs is close to the 10+ yrs asked for. Main gap disclosed honestly: role is a formal pre-sales/post-sales solutions-consulting seat with external enterprise customers -- Siva's stakeholder work has been internal only, even though he owns TokenSight end to end. Listing does not confirm remote-from-India eligibility or visa sponsorship (SingleStore has a Bangalore office but this req is listed under US salary bands) -- flagged in cover letter.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Revin</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Senior/ Staff Product Engineer (Full Stack)</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>JOBSEARCH_105065</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Indeed (API)</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>New York, NY (on-site, 4 days/week)</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>https://to.indeed.com/aaxfbtbmpdd6</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>78% Fit</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Ready to Apply</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr">
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr">
         <is>
           <t>Strong match: TypeScript/React fluency and end-to-end AI-powered product ownership (TokenSight: backend + FastAPI/ClickHouse + React/Next.js dashboards, measured via usage/cost metrics) map directly onto this product-engineer role's core ask. 9 yrs fits their Senior/Staff band. Gaps disclosed honestly: TokenSight's users are internal stakeholders, not external paying customers, and the home-services/vertical-SaaS domain is new. Role is on-site in NYC 4 days/week -- relocation and work-authorization/visa sponsorship from India is unconfirmed in the posting, flagged clearly in the cover letter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Keeper Security, Inc.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Senior Software Architect, Security Platform</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_105227</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Remote (US-based company, remote role)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aabnrqymr8cl</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>65% Fit ⚠️</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Strong full-stack-architecture overlap: TokenSight ownership (FastAPI/ClickHouse/Redis backend + React/Next.js frontend, OpenTelemetry tracing, Presidio guardrails) maps directly onto the role's cross-stack architecture ask, and the JD explicitly wants daily Claude/Copilot users, which Siva is. 10+ yrs requested, Siva has 9. MAJOR GAPS disclosed honestly: no formal 'Architect' title or cross-product-line scope, and domain has been AI infrastructure/observability rather than cybersecurity/PAM/zero-trust specifically -- though TokenSight's PII-redaction and guardrails work is a reasonable security-adjacent analogue. Fully remote per posting, no relocation needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>G-P (Globalization Partners)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Principal Software Engineer - Marketing Technology (Agentic AI)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>JOBSEARCH_105228</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Indeed (API)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aasfjdl7jwmy</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>70% Fit</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Ready to Apply</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Strong stack match: React/Next.js + Python/Node backend is an exact fit, and hands-on production LLM work (TokenSight: multi-provider API integration, prompt-level cost optimization, Presidio guardrails, OpenTelemetry tracing) directly covers the role's 'architect production-grade agentic AI systems' ask. 8+ yrs clears easily with 9. MAJOR GAPS disclosed honestly: no hands-on experience with named agent-orchestration frameworks (LangGraph/CrewAI/AutoGen) -- Siva's tool-calling work has been built directly against provider APIs -- and no MarTech/CRM integration background (Salesforce, HubSpot). Posting lists Boston, MA with no remote-from-India eligibility or visa sponsorship addressed -- flagged clearly as an open question before applying, not assumed either way.</t>
         </is>
       </c>
     </row>

</xml_diff>